<commit_message>
Implement PDF generation service and update related build configurations
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/reports/exports/reportes-ventas-normal-global.xlsx
+++ b/reports/exports/reportes-ventas-normal-global.xlsx
@@ -32,12 +32,39 @@
     <sheet sheetId="26" name="Grafico X04 · Participación Glo" state="visible" r:id="rId29"/>
     <sheet sheetId="27" name="Grafico X04 · Mezcla de Pago (T" state="visible" r:id="rId30"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Día'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Día de semana'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Hora'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Sitio'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Producto'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Tela'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Color'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Vendedor'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Cliente'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'Forma de pago'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'Estado de factura'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="13">'Mejores productos'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="14">'Peores productos'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="15">'Clasificación ABC'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="16">'Pares de productos en canasta'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="17">'Resumen de cancelaciones'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="18">'Cancelaciones'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="19">'Productos cancelados'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="20">'X04 · Tabla comparativa por tie'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="21">'Grafico Ventas diarias'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="22">'Grafico Ventas por hora'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="23">'Grafico Ventas por día'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="24">'Grafico X04 · Ventas por Tienda'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="25">'Grafico X04 · Participación Glo'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="26">'Grafico X04 · Mezcla de Pago (T'!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="114">
   <si>
     <t>Reporte</t>
   </si>
@@ -48,25 +75,37 @@
     <t>Generado</t>
   </si>
   <si>
-    <t>2026-09-15T00:15:46.072Z</t>
+    <t>14 de septiembre de 2026, 8:02 p.m.</t>
   </si>
   <si>
     <t>Periodo</t>
   </si>
   <si>
-    <t>{"desde":"2026-01-01T06:00:00.000Z","hasta":"2027-01-01T05:59:59.999Z","previousDesde":"2025-01-01T06:00:00.000Z","previousHasta":"2026-01-01T05:59:59.999Z","yearAgoDesde":"2025-01-01T06:00:00.000Z","yearAgoHasta":"2026-01-01T05:59:59.999Z"}</t>
+    <t>Del 1 de enero al 31 de diciembre de 2026</t>
   </si>
   <si>
     <t>Filtros</t>
   </si>
   <si>
-    <t>["periodo=personalizado","desde=2026-01-01","hasta=2026-12-31","modalidad=TODO","margenUmbral=15","coberturaCritico=7","coberturaBajo=15","coberturaNormal=60","coberturaExceso=90","modo=normal","umbralCorte=0","umbralTienda=0","agrupacion=semana"]</t>
+    <t xml:space="preserve">Periodo: Personalizado
+Desde: 1 de enero de 2026
+Hasta: 31 de diciembre de 2026
+Modalidad: Todas las modalidades
+Umbral de margen: 15
+Cobertura crítica: 7
+Cobertura baja: 15
+Cobertura normal: 60
+Cobertura exceso: 90
+Modo: Normal
+Umbral de corte: 0
+Umbral de tienda: 0
+Agrupación: semana</t>
   </si>
   <si>
     <t>Modalidad</t>
   </si>
   <si>
-    <t>TODO</t>
+    <t>Todas las modalidades</t>
   </si>
   <si>
     <t>Indicador</t>
@@ -150,6 +189,9 @@
     <t>2026-09-13</t>
   </si>
   <si>
+    <t>Total general</t>
+  </si>
+  <si>
     <t>Día de semana</t>
   </si>
   <si>
@@ -354,34 +396,19 @@
     <t>Total General</t>
   </si>
   <si>
-    <t>100.00</t>
-  </si>
-  <si>
-    <t>103302.00</t>
-  </si>
-  <si>
-    <t>16480.00</t>
-  </si>
-  <si>
-    <t>25825.50</t>
-  </si>
-  <si>
     <t>Rollos · metros: 4986.000 · Rollos · kilos: 0.000 · Rollos · bolsas: 0.000 · Metraje · metros: 0.000 · Metraje · bolsas: 0.000</t>
   </si>
   <si>
     <t>Efectivo: 103302.00 · Transferencia: 0.00 · Crédito: 0.00</t>
   </si>
   <si>
-    <t>0.00</t>
-  </si>
-  <si>
-    <t>dimension</t>
-  </si>
-  <si>
-    <t>fecha</t>
-  </si>
-  <si>
-    <t>nombreUbicacion</t>
+    <t>Dimension</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Nombre Ubicacion</t>
   </si>
   <si>
     <t>Efectivo</t>
@@ -397,10 +424,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -408,13 +436,30 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2F0D9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -429,12 +474,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -776,44 +852,48 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100" style="2" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -825,63 +905,66 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -889,37 +972,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4430</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>85510</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>71810</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>13700</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>16.021517951116827</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -927,118 +1010,126 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>556</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>1</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>17792</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>15012</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>2780</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="G4" s="3">
+    <row r="4" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="15">
         <v>4986</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1">
+      <c r="H4" s="14"/>
+      <c r="I4" s="16">
         <v>103302</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="16">
         <v>86822</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="16">
         <v>16480</v>
       </c>
-      <c r="L4" s="4"/>
+      <c r="L4" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -1046,171 +1137,185 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4986</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>4</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>103302</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>86822</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>16480</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.95322452614664</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="G3" s="3">
+    <row r="3" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="15">
         <v>4986</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="1">
+      <c r="H3" s="14"/>
+      <c r="I3" s="16">
         <v>103302</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="16">
         <v>86822</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="16">
         <v>16480</v>
       </c>
-      <c r="L3" s="4"/>
+      <c r="L3" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14" style="2" customWidth="1"/>
-    <col min="4" max="4" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="5" customWidth="1"/>
+    <col min="4" max="4" width="30" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:4" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>64</v>
+      <c r="D1" s="11" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="5">
         <v>4</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="4">
         <v>103302</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C3" s="2"/>
-      <c r="D3" s="1">
+    <row r="3" spans="1:4" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="16">
         <v>103302</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -1218,118 +1323,126 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4986</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>4</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>103302</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>86822</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>16480</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.95322452614664</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="G3" s="3">
+    <row r="3" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="15">
         <v>4986</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="1">
+      <c r="H3" s="14"/>
+      <c r="I3" s="16">
         <v>103302</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="16">
         <v>86822</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="16">
         <v>16480</v>
       </c>
-      <c r="L3" s="4"/>
+      <c r="L3" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -1337,37 +1450,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>1887</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>1</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>60384</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>50949</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>9435</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -1375,37 +1488,37 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>849</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>27168</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>22923</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>4245</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -1413,37 +1526,37 @@
       <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>1750</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="5">
         <v>1</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="4">
         <v>12250</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="4">
         <v>10150</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="4">
         <v>2100</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="7">
         <v>17.142857142857142</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -1451,110 +1564,102 @@
       <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>500</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="5">
         <v>1</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="4">
         <v>3500</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="4">
         <v>2800</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="4">
         <v>700</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="7">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -1562,37 +1667,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>500</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>1</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>3500</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>2800</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>700</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -1600,37 +1705,37 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>1750</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>1</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>12250</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>10150</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>2100</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>17.142857142857142</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -1638,37 +1743,37 @@
       <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>849</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="5">
         <v>2</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="4">
         <v>27168</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="4">
         <v>22923</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="4">
         <v>4245</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -1676,85 +1781,77 @@
       <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>1887</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="5">
         <v>1</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="4">
         <v>60384</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="4">
         <v>50949</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="4">
         <v>9435</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="7">
         <v>15.625</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="4"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="14" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14" style="4" customWidth="1"/>
+    <col min="5" max="5" width="14" style="7" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F1" t="s">
+      <c r="E1" s="12" t="s">
         <v>70</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -1762,19 +1859,19 @@
       <c r="C2" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="4">
         <v>60384</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="7">
         <v>58.453853749201365</v>
       </c>
       <c r="F2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -1782,19 +1879,19 @@
       <c r="C3" t="s">
         <v>35</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="4">
         <v>27168</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="7">
         <v>84.75344136609165</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -1802,19 +1899,19 @@
       <c r="C4" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="4">
         <v>12250</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="7">
         <v>96.61187585913147</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -1822,157 +1919,147 @@
       <c r="C5" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="4">
         <v>3500</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="7">
         <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D6" s="1"/>
-      <c r="E6" s="4"/>
+        <v>74</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F3"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D1" t="s">
+      <c r="C1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="D1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
         <v>33</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="5">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E3" s="2"/>
+        <v>79</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="21" style="2" customWidth="1"/>
-    <col min="3" max="3" width="21" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21" style="5" customWidth="1"/>
+    <col min="3" max="3" width="21" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B2" s="2"/>
-      <c r="C2" s="1"/>
+      <c r="C1" s="11" t="s">
+        <v>81</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F2"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="14" style="2" customWidth="1"/>
-    <col min="6" max="6" width="21" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="5" customWidth="1"/>
+    <col min="6" max="6" width="21" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:6" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="E2" s="2"/>
-      <c r="F2" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
@@ -1985,11 +2072,11 @@
     <col min="2" max="2" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1997,7 +2084,7 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="4">
         <v>103302</v>
       </c>
     </row>
@@ -2005,7 +2092,7 @@
       <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="5">
         <v>4</v>
       </c>
     </row>
@@ -2013,7 +2100,7 @@
       <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="4">
         <v>103302</v>
       </c>
     </row>
@@ -2021,7 +2108,7 @@
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="5">
         <v>4</v>
       </c>
     </row>
@@ -2029,7 +2116,7 @@
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="4">
         <v>25825.5</v>
       </c>
     </row>
@@ -2037,7 +2124,7 @@
       <c r="A7" t="s">
         <v>17</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="4">
         <v>0</v>
       </c>
     </row>
@@ -2045,7 +2132,7 @@
       <c r="A8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="5">
         <v>0</v>
       </c>
     </row>
@@ -2053,7 +2140,7 @@
       <c r="A9" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="4">
         <v>0</v>
       </c>
     </row>
@@ -2061,7 +2148,7 @@
       <c r="A10" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="6">
         <v>4986</v>
       </c>
     </row>
@@ -2073,295 +2160,300 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="14" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F2" s="2"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="1"/>
+      <c r="H1" s="11" t="s">
+        <v>86</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="14" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14" style="4" customWidth="1"/>
-    <col min="5" max="5" width="14" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="7" customWidth="1"/>
+    <col min="3" max="3" width="14" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14" style="7" customWidth="1"/>
+    <col min="5" max="5" width="14" style="4" customWidth="1"/>
+    <col min="6" max="6" width="14" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14" style="4" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="19" customWidth="1"/>
-    <col min="11" max="11" width="14" style="4" customWidth="1"/>
-    <col min="12" max="12" width="14" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="7" customWidth="1"/>
+    <col min="12" max="12" width="14" style="4" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="4" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:13" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="B1" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="G1" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="I1" t="s">
+      <c r="H1" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="J1" t="s">
+      <c r="I1" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="J1" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="K1" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="M1" t="s">
+      <c r="L1" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="M1" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="4">
+        <v>45</v>
+      </c>
+      <c r="B2" s="7">
         <v>17.22</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="4">
         <v>17792</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="7">
         <v>100</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="4">
         <v>2780</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="5">
         <v>1</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="4">
         <v>17792</v>
       </c>
       <c r="H2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J2" t="s">
-        <v>97</v>
-      </c>
-      <c r="K2" s="4">
-        <v>0</v>
-      </c>
-      <c r="L2" s="1">
+        <v>98</v>
+      </c>
+      <c r="K2" s="7">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4">
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B3" s="4">
-        <v>0</v>
-      </c>
-      <c r="C3" s="1">
-        <v>0</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0</v>
-      </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
+        <v>99</v>
+      </c>
+      <c r="B3" s="7">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="7">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4">
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I3" t="s">
-        <v>100</v>
-      </c>
-      <c r="K3" s="4">
-        <v>0</v>
-      </c>
-      <c r="L3" s="1">
+        <v>101</v>
+      </c>
+      <c r="K3" s="7">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4">
         <v>0</v>
       </c>
       <c r="M3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="4">
+        <v>44</v>
+      </c>
+      <c r="B4" s="7">
         <v>82.78</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="4">
         <v>85510</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="7">
         <v>100</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="4">
         <v>13700</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="5">
         <v>3</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4" s="4">
         <v>28503.33</v>
       </c>
       <c r="H4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J4" t="s">
-        <v>103</v>
-      </c>
-      <c r="K4" s="4">
-        <v>0</v>
-      </c>
-      <c r="L4" s="1">
+        <v>104</v>
+      </c>
+      <c r="K4" s="7">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4">
         <v>0</v>
       </c>
       <c r="M4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="B5" s="17">
+        <v>100</v>
+      </c>
+      <c r="C5" s="16">
+        <v>103302</v>
+      </c>
+      <c r="D5" s="17"/>
+      <c r="E5" s="16">
+        <v>16480</v>
+      </c>
+      <c r="F5" s="14">
+        <v>4</v>
+      </c>
+      <c r="G5" s="16">
+        <v>25825.5</v>
+      </c>
+      <c r="H5" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="1" t="s">
+      <c r="I5" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="F5" s="2">
-        <v>4</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="H5" t="s">
-        <v>109</v>
-      </c>
-      <c r="I5" t="s">
-        <v>110</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>111</v>
-      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="17">
+        <v>0</v>
+      </c>
+      <c r="L5" s="16">
+        <v>0</v>
+      </c>
+      <c r="M5" s="13"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" t="s">
-        <v>68</v>
+    <row r="1" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="4">
         <v>93926</v>
       </c>
     </row>
@@ -2369,117 +2461,127 @@
       <c r="A3" t="s">
         <v>36</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <v>9376</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" t="s">
-        <v>68</v>
+    <row r="1" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2">
+        <v>42</v>
+      </c>
+      <c r="B2" s="4">
         <v>103302</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" t="s">
-        <v>68</v>
+    <row r="1" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2">
+        <v>39</v>
+      </c>
+      <c r="B2" s="4">
         <v>93926</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3">
+        <v>40</v>
+      </c>
+      <c r="B3" s="4">
         <v>9376</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="4" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="4" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" s="19" t="s">
         <v>44</v>
-      </c>
-      <c r="C1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="4">
         <v>17792</v>
       </c>
-      <c r="D2">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4">
         <v>76134</v>
       </c>
     </row>
@@ -2487,192 +2589,200 @@
       <c r="A3" t="s">
         <v>36</v>
       </c>
-      <c r="D3">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4">
         <v>9376</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B1" t="s">
-        <v>68</v>
+    <row r="1" spans="1:2" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2">
+        <v>45</v>
+      </c>
+      <c r="B2" s="4">
         <v>17792</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B3">
+        <v>99</v>
+      </c>
+      <c r="B3" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4">
+        <v>44</v>
+      </c>
+      <c r="B4" s="4">
         <v>85510</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="3" width="16" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D1" t="s">
-        <v>117</v>
+    <row r="1" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2">
+        <v>45</v>
+      </c>
+      <c r="B2" s="4">
         <v>17792</v>
       </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+      <c r="D2" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
+        <v>99</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4">
+        <v>44</v>
+      </c>
+      <c r="B4" s="4">
         <v>85510</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2686,31 +2796,31 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4693</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>93926</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>78911</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>15015</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.985988970040243</v>
       </c>
     </row>
@@ -2724,119 +2834,127 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>293</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>1</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>9376</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>7911</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>1465</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="G4" s="3">
+    <row r="4" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="15">
         <v>4986</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1">
+      <c r="H4" s="14"/>
+      <c r="I4" s="16">
         <v>103302</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="16">
         <v>86822</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="16">
         <v>16480</v>
       </c>
-      <c r="L4" s="4"/>
+      <c r="L4" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -2844,37 +2962,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4693</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>93926</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>78911</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>15015</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.985988970040243</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -2882,118 +3000,126 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>293</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>1</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>9376</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>7911</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>1465</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="G4" s="3">
+    <row r="4" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="15">
         <v>4986</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1">
+      <c r="H4" s="14"/>
+      <c r="I4" s="16">
         <v>103302</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="16">
         <v>86822</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="16">
         <v>16480</v>
       </c>
-      <c r="L4" s="4"/>
+      <c r="L4" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -3001,118 +3127,126 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4986</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>4</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>103302</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>86822</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>16480</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.95322452614664</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="G3" s="3">
+    <row r="3" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="15">
         <v>4986</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="1">
+      <c r="H3" s="14"/>
+      <c r="I3" s="16">
         <v>103302</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="16">
         <v>86822</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="16">
         <v>16480</v>
       </c>
-      <c r="L3" s="4"/>
+      <c r="L3" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -3120,37 +3254,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>4430</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>85510</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>71810</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>13700</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>16.021517951116827</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -3158,118 +3292,126 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>556</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>1</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>17792</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>15012</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>2780</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="G4" s="3">
+    <row r="4" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="15">
         <v>4986</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1">
+      <c r="H4" s="14"/>
+      <c r="I4" s="16">
         <v>103302</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="16">
         <v>86822</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="16">
         <v>16480</v>
       </c>
-      <c r="L4" s="4"/>
+      <c r="L4" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -3277,37 +3419,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>1887</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>1</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>60384</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>50949</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>9435</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -3315,37 +3457,37 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>849</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>27168</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>22923</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>4245</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -3353,37 +3495,37 @@
       <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>1750</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="5">
         <v>1</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="4">
         <v>12250</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="4">
         <v>10150</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="4">
         <v>2100</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="7">
         <v>17.142857142857142</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -3391,118 +3533,126 @@
       <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>500</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="5">
         <v>1</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="4">
         <v>3500</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="4">
         <v>2800</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="4">
         <v>700</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="7">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="G6" s="3">
+    <row r="6" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="15">
         <v>4986</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="1">
+      <c r="H6" s="14"/>
+      <c r="I6" s="16">
         <v>103302</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="16">
         <v>86822</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="16">
         <v>16480</v>
       </c>
-      <c r="L6" s="4"/>
+      <c r="L6" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -3510,37 +3660,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>2736</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>3</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>87552</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>73872</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>13680</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -3548,118 +3698,126 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>2250</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>15750</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>12950</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>2800</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>17.77777777777778</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="G4" s="3">
+    <row r="4" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="15">
         <v>4986</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="1">
+      <c r="H4" s="14"/>
+      <c r="I4" s="16">
         <v>103302</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="16">
         <v>86822</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="16">
         <v>16480</v>
       </c>
-      <c r="L4" s="4"/>
+      <c r="L4" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="19" customWidth="1"/>
-    <col min="4" max="4" width="35" style="2" customWidth="1"/>
-    <col min="5" max="5" width="42" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35" style="5" customWidth="1"/>
+    <col min="5" max="5" width="42" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="14" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14" style="2" customWidth="1"/>
-    <col min="9" max="9" width="19" style="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" style="4" customWidth="1"/>
+    <col min="7" max="7" width="14" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14" style="5" customWidth="1"/>
+    <col min="9" max="9" width="19" style="4" customWidth="1"/>
+    <col min="10" max="10" width="18" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:12" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="12" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
         <v>33</v>
@@ -3667,37 +3825,37 @@
       <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="2">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="D2" s="5">
+        <v>0</v>
+      </c>
+      <c r="E2" s="5">
         <v>0</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>1887</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="5">
         <v>1</v>
       </c>
-      <c r="I2" s="1">
+      <c r="I2" s="4">
         <v>60384</v>
       </c>
-      <c r="J2" s="1">
+      <c r="J2" s="4">
         <v>50949</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="4">
         <v>9435</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
         <v>33</v>
@@ -3705,37 +3863,37 @@
       <c r="C3" t="s">
         <v>34</v>
       </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="D3" s="5">
+        <v>0</v>
+      </c>
+      <c r="E3" s="5">
         <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>849</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="5">
         <v>2</v>
       </c>
-      <c r="I3" s="1">
+      <c r="I3" s="4">
         <v>27168</v>
       </c>
-      <c r="J3" s="1">
+      <c r="J3" s="4">
         <v>22923</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="4">
         <v>4245</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="7">
         <v>15.625</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
         <v>33</v>
@@ -3743,37 +3901,37 @@
       <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="2">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2">
+      <c r="D4" s="5">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0</v>
       </c>
       <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>1750</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="5">
         <v>1</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I4" s="4">
         <v>12250</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="4">
         <v>10150</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="4">
         <v>2100</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="7">
         <v>17.142857142857142</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
         <v>33</v>
@@ -3781,55 +3939,60 @@
       <c r="C5" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="D5" s="5">
+        <v>0</v>
+      </c>
+      <c r="E5" s="5">
         <v>0</v>
       </c>
       <c r="F5" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>500</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="5">
         <v>1</v>
       </c>
-      <c r="I5" s="1">
+      <c r="I5" s="4">
         <v>3500</v>
       </c>
-      <c r="J5" s="1">
+      <c r="J5" s="4">
         <v>2800</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="4">
         <v>700</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="7">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="G6" s="3">
+    <row r="6" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="15">
         <v>4986</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="1">
+      <c r="H6" s="14"/>
+      <c r="I6" s="16">
         <v>103302</v>
       </c>
-      <c r="J6" s="1">
+      <c r="J6" s="16">
         <v>86822</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="16">
         <v>16480</v>
       </c>
-      <c r="L6" s="4"/>
+      <c r="L6" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>